<commit_message>
docs: doi ngay giai doan sang ngay that tinh tu 03/07/2026
</commit_message>
<xml_diff>
--- a/Task_Tracker.xlsx
+++ b/Task_Tracker.xlsx
@@ -615,7 +615,7 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="C4" s="23" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="B5" s="23" t="inlineStr">
         <is>
-          <t>Ngày 7-10</t>
+          <t>09/07 - 12/07/2026</t>
         </is>
       </c>
       <c r="C5" s="23" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E2" s="9" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -1070,7 +1070,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Ngày 7-10</t>
+          <t>09/07 - 12/07/2026</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Ngày 7-10</t>
+          <t>09/07 - 12/07/2026</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Ngày 11-18</t>
+          <t>13/07 - 20/07/2026</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Ngày 1-6</t>
+          <t>03/07 - 08/07/2026</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">

</xml_diff>